<commit_message>
Portal: popis portalu, uprava scenaru
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2114,12 +2114,12 @@
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>V repu je jen požadavky + matice oprávnění; popis portálu (15_Webovy_portal_popis.docx) chybí – nahrát. Nesoulad: Ema dává pacientovi GET /alerty, matice portálu ne – sjednotit.</t>
+          <t>Popis portálu v Sabi/15_Webovy_portal_popis.docx. Oprávnění pacienta k alertům sladí Ema v API (viz Vzkazy).</t>
         </is>
       </c>
       <c r="H19" s="13">
@@ -4892,7 +4892,7 @@
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G79" s="10" t="n"/>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G81" s="10" t="n"/>
@@ -4970,14 +4970,10 @@
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
-        </is>
-      </c>
-      <c r="G82" s="10" t="inlineStr">
-        <is>
-          <t>Popis portálu nahrát do repa.</t>
-        </is>
-      </c>
+          <t>Hotovo</t>
+        </is>
+      </c>
+      <c r="G82" s="10" t="n"/>
     </row>
     <row r="83" ht="42.75" customHeight="1">
       <c r="A83" s="15" t="n">

</xml_diff>

<commit_message>
Testovani: navrh kapitoly s typy testu a scenari
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2188,12 +2188,12 @@
       </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Podklady už existují: testy T01–T10 (Maky/04) a testovací scénáře API (Ema/Implementace §7).</t>
+          <t>Návrh v Sabi/17_Testovani.docx (~2,5 strany). Zbývá: scénáře A-, S- a I- odsouhlasit s Maky, Emou a rolí 4.</t>
         </is>
       </c>
       <c r="H21" s="13">
@@ -5108,7 +5108,7 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G87" s="10" t="n"/>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="F88" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G88" s="10" t="n"/>
@@ -5160,10 +5160,14 @@
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G89" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G89" s="10" t="inlineStr">
+        <is>
+          <t>Scénáře převzaty z Maky/04 a Ema/Implementace §7; integrátor navržen – ověřit.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="7" t="n">
@@ -5186,7 +5190,7 @@
       </c>
       <c r="F90" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G90" s="10" t="n"/>
@@ -5212,7 +5216,7 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G91" s="10" t="n"/>
@@ -5238,7 +5242,7 @@
       </c>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G92" s="10" t="n"/>

</xml_diff>

<commit_message>
Spolecne pozadavky: sloucena tabulka FP/NFP, vzkaz k odsouhlaseni
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -1638,7 +1638,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Požadavky mají zatím jen role 1 (M-F01–10) a role 2 (FP-P01–11); role 3 a 4 chybí. Sjednotit prefixy (M-F vs FP-A), spojit do jedné tabulky, MoSCoW. Chybí: průvodce měřením, připomínky, nepravidelný rytmus, doporučení lékaře v aplikaci.</t>
+          <t>Spojeno do spolecny/Pozadavky_spolecne.xlsx (46 FP + 17 NFP, MoSCoW). Čeká na odsouhlasení vlastníky bloků do 1. 11., pak kapitola (Sabi).</t>
         </is>
       </c>
       <c r="H6" s="13">
@@ -3048,10 +3048,14 @@
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
-        </is>
-      </c>
-      <c r="G11" s="10" t="n"/>
+          <t>Hotovo</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Ve společné tabulce; čeká na potvrzení</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="A12" s="15" t="n">
@@ -3074,10 +3078,14 @@
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
-        </is>
-      </c>
-      <c r="G12" s="10" t="n"/>
+          <t>Hotovo</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Ve společné tabulce; čeká na potvrzení</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="28.5" customHeight="1">
       <c r="A13" s="15" t="n">
@@ -3100,10 +3108,14 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G13" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Očíslováno, MoSCoW navrženo – odsouhlasit</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">

</xml_diff>

<commit_message>
Portal: navrh GUI (7 obrazovek), pripominky k navrhu aplikace
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2151,12 +2151,12 @@
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Počkat na vzhled aplikace (Maky) – sjednotit barvy.</t>
+          <t>7 obrazovek v Sabi/GUI_portal + popis v Sabi/16_GUI_portal.docx, barvy podle návrhu Maky. Zbývá odsouhlasit s Maky (jednotný styl, barevné indikátory).</t>
         </is>
       </c>
       <c r="H20" s="13">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G83" s="10" t="n"/>
@@ -5038,10 +5038,14 @@
       </c>
       <c r="F84" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G84" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>Barvy převzaty od Maky; sladit indikátory hodnot</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="15" t="n">
@@ -5064,7 +5068,7 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G85" s="10" t="n"/>
@@ -5090,7 +5094,7 @@
       </c>
       <c r="F86" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G86" s="10" t="n"/>

</xml_diff>

<commit_message>
Role 4: stavovy diagram synchronizace s NIS a popis
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -541,7 +541,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Domi (možná převezme Sabi – upřesnit)</t>
+          <t>Sabi (převzala roli 4 od Domi 30. 10.) – výstupy v Role4-S</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1382,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Maky = 1, Sabi = 2, Ema = 3, Domi = 4</t>
+          <t>Maky = 1, Sabi = 2 i 4, Ema = 3</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -1457,12 +1457,12 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Domi zatím nic; možná převezme Sabi – rozhodnout v týmu a promítnout do výkazu práce</t>
+          <t>Roli 4 dělá Sabi (od 30. 10.), výstupy ve složce Role4-S; promítnout do výkazu práce a říct cvičícím 12. 11.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Otevřené</t>
+          <t>Vyřešeno</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2406,7 @@
         </is>
       </c>
       <c r="E27" s="12" t="n">
-        <v>46323</v>
+        <v>46330</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
@@ -2415,7 +2415,7 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Role 4 – složka Domi je zatím prázdná.</t>
+          <t>Sabi (role 4). Posunuto z 28. 10. – potřeba na konzultaci 12. 11.</t>
         </is>
       </c>
       <c r="H27" s="13">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Role 4 – podklad: tabulka NisSynchronizace v ER Emy.</t>
+          <t>Diagram (8 stavů) + popis v Role4-S. Zbývá: export PNG z draw.io a potvrdit s Emou hodnoty NisSynchronizace.stav (čeká / odesláno / chyba).</t>
         </is>
       </c>
       <c r="H28" s="13">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Role 4.</t>
+          <t>Sabi (role 4). Sladit s ER Emy (NisSynchronizace) a LOINC kódy.</t>
         </is>
       </c>
       <c r="H29" s="13">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Role 4 – termín 18.11.; zdroje ESH už jsou připravené (Sabi).</t>
+          <t>Sabi (role 4). Zdroje ESH už připravené.</t>
         </is>
       </c>
       <c r="H30" s="13">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Role 4.</t>
+          <t>Sabi (role 4) – případně nabídnout Emě (souvisí se serverem).</t>
         </is>
       </c>
       <c r="H31" s="13">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G124" s="10" t="n"/>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G125" s="10" t="n"/>
@@ -6186,10 +6186,14 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G126" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G126" s="10" t="inlineStr">
+        <is>
+          <t>Diagram + popis hotové, chybí export PNG</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="7" t="n">

</xml_diff>

<commit_message>
Role 4: use case diagram integratoru a popis
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2410,12 +2410,12 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Sabi (role 4). Posunuto z 28. 10. – potřeba na konzultaci 12. 11.</t>
+          <t>Diagram + popis v Role4-S (Administrátor 5 UC, NIS 4 UC, Časovač). Zbývá export PNG z draw.io.</t>
         </is>
       </c>
       <c r="H27" s="13">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Diagram (8 stavů) + popis v Role4-S. Zbývá: export PNG z draw.io a potvrdit s Emou hodnoty NisSynchronizace.stav (čeká / odesláno / chyba).</t>
+          <t>Diagram, PNG (SD_synchronizace.drawio.png) a popis v Role4-S. Zbývá jen potvrdit s Emou hodnoty NisSynchronizace.stav (čeká / odesláno / chyba).</t>
         </is>
       </c>
       <c r="H28" s="13">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G120" s="10" t="n"/>
@@ -6052,7 +6052,7 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G121" s="10" t="n"/>
@@ -6078,10 +6078,14 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G122" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G122" s="10" t="inlineStr">
+        <is>
+          <t>Chybí export PNG</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n">
@@ -6104,7 +6108,7 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G123" s="10" t="n"/>
@@ -6186,14 +6190,10 @@
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
-        </is>
-      </c>
-      <c r="G126" s="10" t="inlineStr">
-        <is>
-          <t>Diagram + popis hotové, chybí export PNG</t>
-        </is>
-      </c>
+          <t>Hotovo</t>
+        </is>
+      </c>
+      <c r="G126" s="10" t="n"/>
     </row>
     <row r="127" ht="30" customHeight="1">
       <c r="A127" s="7" t="n">

</xml_diff>

<commit_message>
Role 4: popis integratoru a FHIR, otazky pro Emu a na konzultaci
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2484,12 +2484,12 @@
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Sabi (role 4). Sladit s ER Emy (NisSynchronizace) a LOINC kódy.</t>
+          <t>Text v Role4-S/25_Integrator_FHIR.docx (mapování, průběh, nastavení, ukázka JSON). Zbývá: potvrdit s Emou NisSynchronizace a práva DB účtu; na konzultaci ověřit hloubku FHIR a FP-I09.</t>
         </is>
       </c>
       <c r="H29" s="13">
@@ -6220,7 +6220,7 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G127" s="10" t="n"/>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G128" s="10" t="n"/>
@@ -6272,10 +6272,14 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G129" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G129" s="10" t="inlineStr">
+        <is>
+          <t>Životospráva do NIS – otevřené (FP-I09)</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="28.5" customHeight="1">
       <c r="A130" s="7" t="n">
@@ -6298,7 +6302,7 @@
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G130" s="10" t="n"/>
@@ -6324,7 +6328,7 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G131" s="10" t="n"/>
@@ -6350,7 +6354,7 @@
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G132" s="10" t="n"/>

</xml_diff>

<commit_message>
Role 4: PNG use case diagramu integratoru
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2410,12 +2410,12 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Diagram + popis v Role4-S (Administrátor 5 UC, NIS 4 UC, Časovač). Zbývá export PNG z draw.io.</t>
+          <t>Role4-S: UC_integrator_NIS.drawio + PNG + popis. Administrátor 5 UC, NIS 4 UC, Časovač.</t>
         </is>
       </c>
       <c r="H27" s="13">
@@ -6078,14 +6078,10 @@
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
-        </is>
-      </c>
-      <c r="G122" s="10" t="inlineStr">
-        <is>
-          <t>Chybí export PNG</t>
-        </is>
-      </c>
+          <t>Hotovo</t>
+        </is>
+      </c>
+      <c r="G122" s="10" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="n">

</xml_diff>

<commit_message>
Role 4: Uvod, vzkaz ke kontrole a dalsi kroky
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -1596,12 +1596,12 @@
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Chybí krok 1.4 – zdůvodnění volby hypertenze do Úvodu (čeká na roli 4).</t>
+          <t>Zdůvodnění volby je v Úvodu (Role4-S/26_Uvod.docx).</t>
         </is>
       </c>
       <c r="H5" s="13">
@@ -2521,12 +2521,12 @@
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Sabi (role 4). Zdroje ESH už připravené.</t>
+          <t>Návrh v Role4-S/26_Uvod.docx (~2,5 str., 9 zdrojů). Zbývá: přečíst týmem, u [4] a [7] ověřit ročník/číslo v originále.</t>
         </is>
       </c>
       <c r="H30" s="13">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G8" s="10" t="n"/>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G133" s="10" t="n"/>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G134" s="10" t="n"/>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G135" s="10" t="n"/>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G136" s="10" t="n"/>
@@ -6484,7 +6484,7 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G137" s="10" t="n"/>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G138" s="10" t="n"/>

</xml_diff>

<commit_message>
Spolecne: Bezpecnost a GDPR, vzkaz ke kontrole
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -1786,7 +1786,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Bezpečnost je rozepsaná v Ema/Implementace §4 a Maky NFR; chybí společná podkapitola a rozhodnutí o retenci dat (GDPR).</t>
+          <t>Návrh podkapitoly v spolecny/06_Bezpecnost_GDPR.docx (Sabi). Zbývá: odsouhlasit týmem, rozhodnout dobu uchování dat (NFP-16), každá role odkáže na podkapitolu ve svém bloku.</t>
         </is>
       </c>
       <c r="H10" s="13">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G31" s="10" t="n"/>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G32" s="10" t="n"/>
@@ -3655,7 +3655,11 @@
           <t>Rozpracováno</t>
         </is>
       </c>
-      <c r="G33" s="10" t="n"/>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Doba uchování – otevřené (NFP-16)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="n">
@@ -3704,10 +3708,14 @@
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G35" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>Podkapitola napsaná; odkazy v blocích doplní každá role</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="7" t="n">

</xml_diff>

<commit_message>
Role 4: Nasazeni, diagram nasazeni, vzkaz pro Emu a Maky
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2558,12 +2558,12 @@
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Rozpracováno</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Sabi (role 4) – případně nabídnout Emě (souvisí se serverem).</t>
+          <t>Návrh v Role4-S/27_Nasazeni.docx + Deployment_diagram.drawio. Zbývá: export PNG, Ema ověří soulad s Implementací (technologie).</t>
         </is>
       </c>
       <c r="H31" s="13">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G139" s="10" t="n"/>
@@ -6574,7 +6574,7 @@
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G140" s="10" t="n"/>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G141" s="10" t="n"/>
@@ -6626,7 +6626,7 @@
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G142" s="10" t="n"/>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G143" s="10" t="n"/>

</xml_diff>

<commit_message>
Spolecne: akteri a rozhrani, vzkaz k odsouhlaseni
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Aktéři jsou v UC diagramech, tok dat v Maky/02-architektura a komponenty v Maky/04. Chybí společné odsouhlasení a role 4.</t>
+          <t>spolecny/03_Akteri_a_rozhrani.docx: aktéři, matice aktér × část, tabulka rozhraní. Zbývá odsouhlasit v týmu.</t>
         </is>
       </c>
       <c r="H7" s="13">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G15" s="10" t="n"/>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G16" s="10" t="n"/>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Rozpracováno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G18" s="10" t="n"/>

</xml_diff>

<commit_message>
Spolecne: navrh kapitoly Analyza pozadavku
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -1638,7 +1638,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>Spojeno do spolecny/Pozadavky_spolecne.xlsx (46 FP + 17 NFP, MoSCoW). Čeká na odsouhlasení vlastníky bloků do 1. 11., pak kapitola (Sabi).</t>
+          <t>Tabulka spolecny/Pozadavky_spolecne.xlsx (čeká na odsouhlasení do 1. 11.) + návrh kapitoly spolecny/02_Analyza_pozadavku.docx (persony, MoSCoW, příloha A). Po odsouhlasení přegenerovat přílohu.</t>
         </is>
       </c>
       <c r="H6" s="13">
@@ -3025,7 +3025,11 @@
           <t>Rozpracováno</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>3 persony v kapitole – odsouhlasit</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="42.75" customHeight="1">
       <c r="A11" s="15" t="n">
@@ -3138,10 +3142,14 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G14" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Návrh kapitoly hotový; čeká na odsouhlasení požadavků</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="7" t="n">

</xml_diff>

<commit_message>
Spolecne: navrh Zhodnoceni, PNG diagramu nasazeni
</commit_message>
<xml_diff>
--- a/Rozdeleni_projektu_SI2.xlsx
+++ b/Rozdeleni_projektu_SI2.xlsx
@@ -2595,10 +2595,14 @@
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G32" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Návrh v spolecny/28_Zhodnoceni.docx (Sabi). Zbývá odsouhlasit v týmu a doladit po konzultaci.</t>
+        </is>
+      </c>
       <c r="H32" s="13">
         <f>COUNTIFS('Osnova kroků'!$A$5:$A$171,A32,'Osnova kroků'!$F$5:$F$171,"Hotovo")&amp;" / "&amp;COUNTIF('Osnova kroků'!$A$5:$A$171,A32)</f>
         <v/>
@@ -6690,7 +6694,7 @@
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G144" s="10" t="n"/>
@@ -6716,7 +6720,7 @@
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G145" s="10" t="n"/>
@@ -6742,7 +6746,7 @@
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
+          <t>Hotovo</t>
         </is>
       </c>
       <c r="G146" s="10" t="n"/>
@@ -6768,10 +6772,14 @@
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t>Nezahájeno</t>
-        </is>
-      </c>
-      <c r="G147" s="10" t="n"/>
+          <t>Rozpracováno</t>
+        </is>
+      </c>
+      <c r="G147" s="10" t="inlineStr">
+        <is>
+          <t>Napsáno, čeká na odsouhlasení</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="7" t="n">

</xml_diff>